<commit_message>
Enhancements to feautres. Analytics, reporting and security rebuilt.
</commit_message>
<xml_diff>
--- a/delete/fee_structures.xlsx
+++ b/delete/fee_structures.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="77">
   <si>
     <t>fee_type</t>
   </si>
@@ -46,76 +46,205 @@
     <t>Transport Fee</t>
   </si>
   <si>
-    <t>Lab Fee</t>
-  </si>
-  <si>
-    <t>Sports Fee</t>
-  </si>
-  <si>
-    <t>Admission Fee</t>
-  </si>
-  <si>
-    <t>Class 10</t>
-  </si>
-  <si>
-    <t>Class 9</t>
-  </si>
-  <si>
-    <t>Class 8</t>
+    <t>Grade 1</t>
+  </si>
+  <si>
+    <t>Grade 2</t>
+  </si>
+  <si>
+    <t>Grade 3</t>
+  </si>
+  <si>
+    <t>Grade 4</t>
+  </si>
+  <si>
+    <t>Grade 5</t>
+  </si>
+  <si>
+    <t>Grade 6</t>
+  </si>
+  <si>
+    <t>Grade 7</t>
+  </si>
+  <si>
+    <t>Grade 8</t>
+  </si>
+  <si>
+    <t>Grade 9</t>
+  </si>
+  <si>
+    <t>Grade 10</t>
+  </si>
+  <si>
+    <t>Grade 11</t>
+  </si>
+  <si>
+    <t>Grade 12</t>
+  </si>
+  <si>
+    <t>3200</t>
+  </si>
+  <si>
+    <t>810</t>
+  </si>
+  <si>
+    <t>3400</t>
+  </si>
+  <si>
+    <t>820</t>
+  </si>
+  <si>
+    <t>3600</t>
+  </si>
+  <si>
+    <t>830</t>
+  </si>
+  <si>
+    <t>3800</t>
+  </si>
+  <si>
+    <t>840</t>
+  </si>
+  <si>
+    <t>4000</t>
+  </si>
+  <si>
+    <t>850</t>
+  </si>
+  <si>
+    <t>4200</t>
+  </si>
+  <si>
+    <t>860</t>
+  </si>
+  <si>
+    <t>4400</t>
+  </si>
+  <si>
+    <t>870</t>
+  </si>
+  <si>
+    <t>4600</t>
+  </si>
+  <si>
+    <t>880</t>
+  </si>
+  <si>
+    <t>4800</t>
+  </si>
+  <si>
+    <t>890</t>
   </si>
   <si>
     <t>5000</t>
   </si>
   <si>
-    <t>1200</t>
-  </si>
-  <si>
-    <t>2000</t>
-  </si>
-  <si>
-    <t>1500</t>
-  </si>
-  <si>
-    <t>8000</t>
+    <t>900</t>
+  </si>
+  <si>
+    <t>5200</t>
+  </si>
+  <si>
+    <t>910</t>
+  </si>
+  <si>
+    <t>5400</t>
+  </si>
+  <si>
+    <t>920</t>
+  </si>
+  <si>
+    <t>TERM</t>
   </si>
   <si>
     <t>MONTHLY</t>
   </si>
   <si>
-    <t>TERM</t>
-  </si>
-  <si>
     <t>YEARLY</t>
   </si>
   <si>
-    <t>ONE_TIME</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
+    <t>15</t>
+  </si>
+  <si>
     <t>true</t>
   </si>
   <si>
     <t>false</t>
   </si>
   <si>
-    <t>Monthly tuition fee</t>
-  </si>
-  <si>
-    <t>Bus transport fee</t>
-  </si>
-  <si>
-    <t>Science lab fee</t>
-  </si>
-  <si>
-    <t>Annual sports fee</t>
-  </si>
-  <si>
-    <t>One-time admission fee</t>
-  </si>
-  <si>
-    <t>2024-25</t>
+    <t>Tuition for Grade 1</t>
+  </si>
+  <si>
+    <t>Transport for Grade 1</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 2</t>
+  </si>
+  <si>
+    <t>Transport for Grade 2</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 3</t>
+  </si>
+  <si>
+    <t>Transport for Grade 3</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 4</t>
+  </si>
+  <si>
+    <t>Transport for Grade 4</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 5</t>
+  </si>
+  <si>
+    <t>Transport for Grade 5</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 6</t>
+  </si>
+  <si>
+    <t>Transport for Grade 6</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 7</t>
+  </si>
+  <si>
+    <t>Transport for Grade 7</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 8</t>
+  </si>
+  <si>
+    <t>Transport for Grade 8</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 9</t>
+  </si>
+  <si>
+    <t>Transport for Grade 9</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 10</t>
+  </si>
+  <si>
+    <t>Transport for Grade 10</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 11</t>
+  </si>
+  <si>
+    <t>Transport for Grade 11</t>
+  </si>
+  <si>
+    <t>Tuition for Grade 12</t>
+  </si>
+  <si>
+    <t>Transport for Grade 12</t>
   </si>
 </sst>
 </file>
@@ -473,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -507,25 +636,22 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="G2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -533,103 +659,528 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="G3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" t="s">
-        <v>33</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" t="s">
-        <v>33</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
-        <v>15</v>
-      </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="F5" t="s">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F12" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" t="s">
+        <v>46</v>
+      </c>
+      <c r="E14" t="s">
+        <v>49</v>
+      </c>
+      <c r="F14" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" t="s">
+        <v>47</v>
+      </c>
+      <c r="E15" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" t="s">
+        <v>49</v>
+      </c>
+      <c r="F16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C18" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" t="s">
+        <v>49</v>
+      </c>
+      <c r="F18" t="s">
+        <v>51</v>
+      </c>
+      <c r="G18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" t="s">
+        <v>52</v>
+      </c>
+      <c r="G19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>40</v>
+      </c>
+      <c r="D20" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" t="s">
+        <v>51</v>
+      </c>
+      <c r="G20" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" t="s">
+        <v>41</v>
+      </c>
+      <c r="D21" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" t="s">
+        <v>52</v>
+      </c>
+      <c r="G21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B22" t="s">
         <v>20</v>
       </c>
-      <c r="D6" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" t="s">
-        <v>33</v>
+      <c r="C22" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" t="s">
+        <v>47</v>
+      </c>
+      <c r="E22" t="s">
+        <v>49</v>
+      </c>
+      <c r="F22" t="s">
+        <v>51</v>
+      </c>
+      <c r="G22" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" t="s">
+        <v>9</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" t="s">
+        <v>47</v>
+      </c>
+      <c r="E23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" t="s">
+        <v>52</v>
+      </c>
+      <c r="G23" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" t="s">
+        <v>47</v>
+      </c>
+      <c r="E24" t="s">
+        <v>49</v>
+      </c>
+      <c r="F24" t="s">
+        <v>51</v>
+      </c>
+      <c r="G24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" t="s">
+        <v>9</v>
+      </c>
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" t="s">
+        <v>47</v>
+      </c>
+      <c r="E25" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" t="s">
+        <v>52</v>
+      </c>
+      <c r="G25" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>